<commit_message>
Implementa plano de decoração + PC sobre a mesa
- PC com gabinete de vidro no canto direito do tampo; remove o suporte suspenso
- Corrige interferência notebook × monitor (monitores 6 cm à esquerda, notebook à frente)
- 3 nichos iluminados sobre a cabeceira, quadros P&B, planta pendente e acessórios
- Validação ampliada: 58/58 verificações OK
- Plantas 2D, orçamento (nichos, LED, decoração estimada), lista de compras gerada por script
- Tour 360° e visualizador 3D atualizados; opções --amostras/--largura nos scripts de render

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M4fUn4zoGcBfLLrM7oKPYT
</commit_message>
<xml_diff>
--- a/PROJETO_QUARTO_ESCRITORIO/04_ORCAMENTO/orcamento_completo.xlsx
+++ b/PROJETO_QUARTO_ESCRITORIO/04_ORCAMENTO/orcamento_completo.xlsx
@@ -42,19 +42,20 @@
     <definedName name="galoes_teto">Quantitativos!$C$29</definedName>
     <definedName name="led_prateleira">Quantitativos!$C$30</definedName>
     <definedName name="led_vertical">Quantitativos!$C$31</definedName>
-    <definedName name="n_verticais">Quantitativos!$C$32</definedName>
-    <definedName name="perda_led">Quantitativos!$C$33</definedName>
-    <definedName name="metros_led">Quantitativos!$C$34</definedName>
-    <definedName name="rolos_led">Quantitativos!$C$35</definedName>
-    <definedName name="barras_perfil">Quantitativos!$C$36</definedName>
-    <definedName name="n_verticais_prem">Quantitativos!$C$37</definedName>
-    <definedName name="metros_led_prem">Quantitativos!$C$38</definedName>
-    <definedName name="rolos_led_prem">Quantitativos!$C$39</definedName>
-    <definedName name="barras_perfil_prem">Quantitativos!$C$40</definedName>
-    <definedName name="contingencia">Quantitativos!$C$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Econômico'!$A$3:$M$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Equilibrado'!$A$3:$M$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Premium'!$A$3:$M$32</definedName>
+    <definedName name="led_nichos">Quantitativos!$C$32</definedName>
+    <definedName name="n_verticais">Quantitativos!$C$33</definedName>
+    <definedName name="perda_led">Quantitativos!$C$34</definedName>
+    <definedName name="metros_led">Quantitativos!$C$35</definedName>
+    <definedName name="rolos_led">Quantitativos!$C$36</definedName>
+    <definedName name="barras_perfil">Quantitativos!$C$37</definedName>
+    <definedName name="n_verticais_prem">Quantitativos!$C$38</definedName>
+    <definedName name="metros_led_prem">Quantitativos!$C$39</definedName>
+    <definedName name="rolos_led_prem">Quantitativos!$C$40</definedName>
+    <definedName name="barras_perfil_prem">Quantitativos!$C$41</definedName>
+    <definedName name="contingencia">Quantitativos!$C$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Econômico'!$A$3:$M$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Equilibrado'!$A$3:$M$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Premium'!$A$3:$M$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -667,7 +668,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B10" s="3">
@@ -684,140 +685,159 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <f>SUMIF('Econômico'!$A:$A,$A11,'Econômico'!$M:$M)</f>
+        <v/>
+      </c>
+      <c r="C11" s="3">
+        <f>SUMIF('Equilibrado'!$A:$A,$A11,'Equilibrado'!$M:$M)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>SUMIF('Premium'!$A:$A,$A11,'Premium'!$M:$M)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Subtotal itens</t>
         </is>
       </c>
-      <c r="B11" s="3">
-        <f>SUM(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="3">
-        <f>SUM(C5:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="3">
-        <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="B12" s="3">
+        <f>SUM(B5:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="3">
+        <f>SUM(C5:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="3">
+        <f>SUM(D5:D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Reserva para imprevistos (10%)</t>
         </is>
       </c>
-      <c r="B12" s="3">
-        <f>B11*contingencia</f>
-        <v/>
-      </c>
-      <c r="C12" s="3">
-        <f>C11*contingencia</f>
-        <v/>
-      </c>
-      <c r="D12" s="3">
-        <f>D11*contingencia</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="B13" s="3">
+        <f>B12*contingencia</f>
+        <v/>
+      </c>
+      <c r="C13" s="3">
+        <f>C12*contingencia</f>
+        <v/>
+      </c>
+      <c r="D13" s="3">
+        <f>D12*contingencia</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="6">
-        <f>B11+B12</f>
-        <v/>
-      </c>
-      <c r="C13" s="6">
-        <f>C11+C12</f>
-        <v/>
-      </c>
-      <c r="D13" s="6">
-        <f>D11+D12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="6">
+        <f>B12+B13</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>C12+C13</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>D12+D13</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>dos quais: preços pesquisados</t>
-        </is>
-      </c>
-      <c r="B15" s="3">
-        <f>SUMIF('Econômico'!$H:$H,"Pesquisado (página do produto)",'Econômico'!$M:$M)+SUMIF('Econômico'!$H:$H,"Pesquisado (listagem da loja)",'Econômico'!$M:$M)</f>
-        <v/>
-      </c>
-      <c r="C15" s="3">
-        <f>SUMIF('Equilibrado'!$H:$H,"Pesquisado (página do produto)",'Equilibrado'!$M:$M)+SUMIF('Equilibrado'!$H:$H,"Pesquisado (listagem da loja)",'Equilibrado'!$M:$M)</f>
-        <v/>
-      </c>
-      <c r="D15" s="3">
-        <f>SUMIF('Premium'!$H:$H,"Pesquisado (página do produto)",'Premium'!$M:$M)+SUMIF('Premium'!$H:$H,"Pesquisado (listagem da loja)",'Premium'!$M:$M)</f>
-        <v/>
-      </c>
+      <c r="A15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>dos quais: preços pesquisados</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <f>SUMIF('Econômico'!$H:$H,"Pesquisado (página do produto)",'Econômico'!$M:$M)+SUMIF('Econômico'!$H:$H,"Pesquisado (listagem da loja)",'Econômico'!$M:$M)</f>
+        <v/>
+      </c>
+      <c r="C16" s="3">
+        <f>SUMIF('Equilibrado'!$H:$H,"Pesquisado (página do produto)",'Equilibrado'!$M:$M)+SUMIF('Equilibrado'!$H:$H,"Pesquisado (listagem da loja)",'Equilibrado'!$M:$M)</f>
+        <v/>
+      </c>
+      <c r="D16" s="3">
+        <f>SUMIF('Premium'!$H:$H,"Pesquisado (página do produto)",'Premium'!$M:$M)+SUMIF('Premium'!$H:$H,"Pesquisado (listagem da loja)",'Premium'!$M:$M)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>dos quais: estimativas</t>
         </is>
       </c>
-      <c r="B16" s="3">
+      <c r="B17" s="3">
         <f>SUMIF('Econômico'!$H:$H,"Estimativa",'Econômico'!$M:$M)</f>
         <v/>
       </c>
-      <c r="C16" s="3">
+      <c r="C17" s="3">
         <f>SUMIF('Equilibrado'!$H:$H,"Estimativa",'Equilibrado'!$M:$M)</f>
         <v/>
       </c>
-      <c r="D16" s="3">
+      <c r="D17" s="3">
         <f>SUMIF('Premium'!$H:$H,"Estimativa",'Premium'!$M:$M)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Notas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>• Piso de madeira colante: fora do orçamento, conforme combinado.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>• Preços Pichau = à vista no PIX. Amazon = preço do anúncio no dia; frete pode variar por CEP.</t>
+          <t>• Piso de madeira colante: fora do orçamento, conforme combinado.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>• Tinta grafite: o preço é o da base branca; a cor preparada em loja pode custar mais. Confirmar na loja.</t>
+          <t>• Preços Pichau = à vista no PIX. Amazon = preço do anúncio no dia; frete pode variar por CEP.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>• Marcenaria (ripado, tampo, prateleira) e mão de obra = estimativas por faixa de mercado; pedir 3 orçamentos locais.</t>
+          <t>• Tinta grafite: o preço é o da base branca; a cor preparada em loja pode custar mais. Confirmar na loja.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>• Marcenaria (ripado, tampo, prateleira) e mão de obra = estimativas por faixa de mercado; pedir 3 orçamentos locais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>• Premium: a estrutura Marsail é vendida pela Amazon Global (importação); prazo e impostos podem variar.</t>
         </is>
@@ -834,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1237,188 +1257,188 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Mobiliário</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Suporte de gabinete</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>C3Tech SC-20BK (piso)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Marcenaria</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Painel ripado Parede D (piso→teto)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Ripado MDF BP amadeirado sobre fundo preto, instalado</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Marceneiro local</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Faixa R$ 250–600/m² instalado (Revista Oeste); R$ 180–750/m² (Monitor do Mercado) — https://monitordomercado.com.br/economia-2/385193-quanto-custa-instalar-painel-ripado-e-transformar-a-sala-com-um-visual-moderno-e-sofisticado/</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>265 × 3 × 264</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>MDF BP</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="14">
+        <f>area_ripado</f>
+        <v/>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="n">
+        <v>250</v>
+      </c>
+      <c r="M9" s="16">
+        <f>J9*L9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Marcenaria</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Prateleiras sobre a mesa</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Prateleira MDF Freijó 80×25 c/ suporte invisível (kit 2)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com.br/dp/B07L41MRLN</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Plástico</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com.br/dp/B0HPF7JM1G</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>2 × (80 × 25)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>MDF freijó</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Pesquisado (listagem da loja)</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="n">
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>32</v>
-      </c>
-      <c r="M9" s="12">
-        <f>J9*L9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>kit</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>436</v>
+      </c>
+      <c r="M10" s="12">
+        <f>J10*L10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Marcenaria</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Painel ripado Parede D (piso→teto)</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Ripado MDF BP amadeirado sobre fundo preto, instalado</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Nichos iluminados 3× (cabeceira)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>MDF BP freijó 15 mm, fundo preto, rasgo p/ LED</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Marceneiro local</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Faixa R$ 250–600/m² instalado (Revista Oeste); R$ 180–750/m² (Monitor do Mercado) — https://monitordomercado.com.br/economia-2/385193-quanto-custa-instalar-painel-ripado-e-transformar-a-sala-com-um-visual-moderno-e-sofisticado/</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>265 × 3 × 264</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>MDF BP</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Estimativa</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
-      <c r="J10" s="14">
-        <f>area_ripado</f>
-        <v/>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="L10" s="15" t="n">
-        <v>250</v>
-      </c>
-      <c r="M10" s="16">
-        <f>J10*L10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Marcenaria</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Prateleiras sobre a mesa</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Prateleira MDF Freijó 80×25 c/ suporte invisível (kit 2)</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com.br/dp/B0HPF7JM1G</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>2 × (80 × 25)</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>MDF freijó</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Pesquisado (listagem da loja)</t>
-        </is>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="n">
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>3 × (24 × 26 × 16)</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>MDF BP freijó</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>kit</t>
-        </is>
-      </c>
-      <c r="L11" s="11" t="n">
-        <v>436</v>
-      </c>
-      <c r="M11" s="12">
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="L11" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="M11" s="16">
         <f>J11*L11</f>
         <v/>
       </c>
@@ -2608,27 +2628,27 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Mão de obra de pintura</t>
+          <t>Luminária de mesa articulada</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Pintor (paredes + teto), sem preparo pesado</t>
+          <t>Luminária articulada preta, E27, lâmpada 2700 K</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Profissional local</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Faixa R$ 15–35/m² simples; R$ 35–60/m² com preparo (Lar Pontual) — https://larpontual.com.br/portal/preco-de-pintor-por-m2</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
@@ -2651,17 +2671,16 @@
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="J31" s="14">
-        <f>area_pintura_total</f>
-        <v/>
+      <c r="J31" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L31" s="15" t="n">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M31" s="16">
         <f>J31*L31</f>
@@ -2671,27 +2690,27 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Frete (itens sem frete grátis)</t>
+          <t>Suporte de headphone</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Reserva de frete</t>
+          <t>Suporte de mesa em metal preto</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Estimativa</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
@@ -2719,78 +2738,574 @@
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L32" s="15" t="n">
-        <v>150</v>
+        <v>42</v>
       </c>
       <c r="M32" s="16">
         <f>J32*L32</f>
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Quadros P&amp;B (3 na parede + 2 na prateleira)</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Impressões P&amp;B 40×55, 2× 36×26, 20×25, 15×20 c/ moldura preta e passe-partout</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L33" s="15" t="n">
+        <v>245</v>
+      </c>
+      <c r="M33" s="16">
+        <f>J33*L33</f>
+        <v/>
+      </c>
+    </row>
     <row r="34">
-      <c r="L34" s="4" t="inlineStr">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Planta pendente</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Vaso cerâmica preta Ø18 + suporte de corda + samambaia + gancho de teto</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J34" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>84</v>
+      </c>
+      <c r="M34" s="16">
+        <f>J34*L34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Objetos dos nichos</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Vaso cerâmica + elefante em madeira + escultura de baleia (~15 cm)</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L35" s="15" t="n">
+        <v>140</v>
+      </c>
+      <c r="M35" s="16">
+        <f>J35*L35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Plantas da prateleira</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Vaso médio c/ planta + suculenta</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J36" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>70</v>
+      </c>
+      <c r="M36" s="16">
+        <f>J36*L36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Relógio LED de prateleira</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Relógio digital LED 12 cm</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J37" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L37" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="M37" s="16">
+        <f>J37*L37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Caneca e acessórios de mesa</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Caneca de cerâmica + porta-lápis</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J38" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="M38" s="16">
+        <f>J38*L38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Mão de obra de pintura</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Pintor (paredes + teto), sem preparo pesado</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Profissional local</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Faixa R$ 15–35/m² simples; R$ 35–60/m² com preparo (Lar Pontual) — https://larpontual.com.br/portal/preco-de-pintor-por-m2</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J39" s="14">
+        <f>area_pintura_total</f>
+        <v/>
+      </c>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="L39" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="M39" s="16">
+        <f>J39*L39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Frete (itens sem frete grátis)</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Reserva de frete</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>150</v>
+      </c>
+      <c r="M40" s="16">
+        <f>J40*L40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="L42" s="4" t="inlineStr">
         <is>
           <t>Subtotal itens</t>
         </is>
       </c>
-      <c r="M34" s="6">
-        <f>SUM(M4:M32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="L35" s="4" t="inlineStr">
+      <c r="M42" s="6">
+        <f>SUM(M4:M40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="L43" s="4" t="inlineStr">
         <is>
           <t>Reserva para imprevistos</t>
         </is>
       </c>
-      <c r="M35" s="6">
-        <f>M34*contingencia</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="L36" s="4" t="inlineStr">
+      <c r="M43" s="6">
+        <f>M42*contingencia</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="L44" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="M36" s="6">
-        <f>M34+M35</f>
+      <c r="M44" s="6">
+        <f>M42+M43</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M32"/>
+  <autoFilter ref="A3:M40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2802,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3205,63 +3720,64 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Mobiliário</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Suporte de gabinete</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Suporte suspenso sob a mesa, giratório (10–15 kg)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com.br/dp/B0GWDYZB8F</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>larg. 13,5–23,5</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Aço</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Pesquisado (listagem da loja)</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>199.49</v>
-      </c>
-      <c r="M9" s="12">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Marcenaria</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Painel ripado Parede D (piso→teto)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Ripado MDF BP freijó + fundo preto, recortes, instalado</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Marceneiro local</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Faixa R$ 250–600/m² instalado (Revista Oeste); R$ 180–750/m² (Monitor do Mercado) — https://monitordomercado.com.br/economia-2/385193-quanto-custa-instalar-painel-ripado-e-transformar-a-sala-com-um-visual-moderno-e-sofisticado/</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>265 × 3 × 264</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>MDF BP freijó</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="14">
+        <f>area_ripado</f>
+        <v/>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="M9" s="16">
         <f>J9*L9</f>
         <v/>
       </c>
@@ -3274,12 +3790,12 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Painel ripado Parede D (piso→teto)</t>
+          <t>Prateleira sobre a mesa</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Ripado MDF BP freijó + fundo preto, recortes, instalado</t>
+          <t>Prateleira freijó 170×25 c/ rasgo para LED, h = 1,95 m</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -3289,12 +3805,12 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Faixa R$ 250–600/m² instalado (Revista Oeste); R$ 180–750/m² (Monitor do Mercado) — https://monitordomercado.com.br/economia-2/385193-quanto-custa-instalar-painel-ripado-e-transformar-a-sala-com-um-visual-moderno-e-sofisticado/</t>
+          <t>Estimativa</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>265 × 3 × 264</t>
+          <t>170 × 25 × 2,5</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
@@ -3312,17 +3828,16 @@
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="J10" s="14">
-        <f>area_ripado</f>
-        <v/>
+      <c r="J10" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L10" s="15" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="M10" s="16">
         <f>J10*L10</f>
@@ -3337,12 +3852,12 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Prateleira sobre a mesa</t>
+          <t>Nichos iluminados 3× (cabeceira)</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>Prateleira freijó 170×25 c/ rasgo para LED, h = 1,95 m</t>
+          <t>MDF BP freijó 15 mm, fundo preto, rasgo p/ LED</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -3357,7 +3872,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>170 × 25 × 2,5</t>
+          <t>3 × (24 × 26 × 16)</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
@@ -3380,11 +3895,11 @@
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>vb</t>
         </is>
       </c>
       <c r="L11" s="15" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="M11" s="16">
         <f>J11*L11</f>
@@ -4514,27 +5029,27 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Mão de obra de pintura</t>
+          <t>Luminária de mesa articulada</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Pintor c/ preparo (paredes + teto)</t>
+          <t>Luminária articulada preta, E27, lâmpada 2700 K</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Profissional local</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Faixa R$ 15–35/m² simples; R$ 35–60/m² com preparo (Lar Pontual) — https://larpontual.com.br/portal/preco-de-pintor-por-m2</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
@@ -4557,17 +5072,16 @@
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="J30" s="14">
-        <f>area_pintura_total</f>
-        <v/>
+      <c r="J30" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L30" s="15" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="M30" s="16">
         <f>J30*L30</f>
@@ -4577,27 +5091,27 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Instalação da iluminação</t>
+          <t>Suporte de headphone</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Montagem das fitas/perfis/fonte (marceneiro ou eletricista)</t>
+          <t>Suporte de mesa em metal preto</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Profissional local</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Estimativa</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
@@ -4625,11 +5139,11 @@
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L31" s="15" t="n">
-        <v>250</v>
+        <v>60</v>
       </c>
       <c r="M31" s="16">
         <f>J31*L31</f>
@@ -4639,27 +5153,27 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Frete (itens sem frete grátis)</t>
+          <t>Quadros P&amp;B (3 na parede + 2 na prateleira)</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Reserva de frete</t>
+          <t>Impressões P&amp;B 40×55, 2× 36×26, 20×25, 15×20 c/ moldura preta e passe-partout</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Estimativa</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
@@ -4687,75 +5201,571 @@
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L32" s="15" t="n">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="M32" s="16">
         <f>J32*L32</f>
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Planta pendente</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Vaso cerâmica preta Ø18 + suporte de corda + samambaia + gancho de teto</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L33" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="M33" s="16">
+        <f>J33*L33</f>
+        <v/>
+      </c>
+    </row>
     <row r="34">
-      <c r="L34" s="4" t="inlineStr">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Objetos dos nichos</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Vaso cerâmica + elefante em madeira + escultura de baleia (~15 cm)</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J34" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="M34" s="16">
+        <f>J34*L34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Plantas da prateleira</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Vaso médio c/ planta + suculenta</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L35" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="M35" s="16">
+        <f>J35*L35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Relógio LED de prateleira</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Relógio digital LED 12 cm</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J36" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>70</v>
+      </c>
+      <c r="M36" s="16">
+        <f>J36*L36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Caneca e acessórios de mesa</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Caneca de cerâmica + porta-lápis</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J37" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L37" s="15" t="n">
+        <v>60</v>
+      </c>
+      <c r="M37" s="16">
+        <f>J37*L37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Mão de obra de pintura</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Pintor c/ preparo (paredes + teto)</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Profissional local</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Faixa R$ 15–35/m² simples; R$ 35–60/m² com preparo (Lar Pontual) — https://larpontual.com.br/portal/preco-de-pintor-por-m2</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J38" s="14">
+        <f>area_pintura_total</f>
+        <v/>
+      </c>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="M38" s="16">
+        <f>J38*L38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Instalação da iluminação</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Montagem das fitas/perfis/fonte (marceneiro ou eletricista)</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Profissional local</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J39" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="L39" s="15" t="n">
+        <v>250</v>
+      </c>
+      <c r="M39" s="16">
+        <f>J39*L39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Frete (itens sem frete grátis)</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Reserva de frete</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="M40" s="16">
+        <f>J40*L40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="L42" s="4" t="inlineStr">
         <is>
           <t>Subtotal itens</t>
         </is>
       </c>
-      <c r="M34" s="6">
-        <f>SUM(M4:M32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="L35" s="4" t="inlineStr">
+      <c r="M42" s="6">
+        <f>SUM(M4:M40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="L43" s="4" t="inlineStr">
         <is>
           <t>Reserva para imprevistos</t>
         </is>
       </c>
-      <c r="M35" s="6">
-        <f>M34*contingencia</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="L36" s="4" t="inlineStr">
+      <c r="M43" s="6">
+        <f>M42*contingencia</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="L44" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="M36" s="6">
-        <f>M34+M35</f>
+      <c r="M44" s="6">
+        <f>M42+M43</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M32"/>
+  <autoFilter ref="A3:M40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4767,7 +5777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5170,63 +6180,64 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Mobiliário</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Suporte de gabinete</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Suporte suspenso sob a mesa, giratório (10–15 kg)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com.br/dp/B0GWDYZB8F</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>larg. 13,5–23,5</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Aço</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Pesquisado (listagem da loja)</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>30/10/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>199.49</v>
-      </c>
-      <c r="M9" s="12">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Marcenaria</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Painel ripado Parede D (piso→teto)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Ripado em lâmina natural freijó + fundo preto, instalado</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Marceneiro local</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Faixa R$ 250–600/m² instalado (Revista Oeste); R$ 180–750/m² (Monitor do Mercado) — https://monitordomercado.com.br/economia-2/385193-quanto-custa-instalar-painel-ripado-e-transformar-a-sala-com-um-visual-moderno-e-sofisticado/</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>265 × 3 × 264</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Lâmina natural</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="14">
+        <f>area_ripado</f>
+        <v/>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="L9" s="15" t="n">
+        <v>600</v>
+      </c>
+      <c r="M9" s="16">
         <f>J9*L9</f>
         <v/>
       </c>
@@ -5239,12 +6250,12 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Painel ripado Parede D (piso→teto)</t>
+          <t>Prateleira sobre a mesa</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Ripado em lâmina natural freijó + fundo preto, instalado</t>
+          <t>Prateleira lâmina natural 170×25 c/ LED embutido, h = 1,95 m</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -5254,12 +6265,12 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>Faixa R$ 250–600/m² instalado (Revista Oeste); R$ 180–750/m² (Monitor do Mercado) — https://monitordomercado.com.br/economia-2/385193-quanto-custa-instalar-painel-ripado-e-transformar-a-sala-com-um-visual-moderno-e-sofisticado/</t>
+          <t>Estimativa</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>265 × 3 × 264</t>
+          <t>170 × 25 × 3</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
@@ -5277,17 +6288,16 @@
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="J10" s="14">
-        <f>area_ripado</f>
-        <v/>
+      <c r="J10" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L10" s="15" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="M10" s="16">
         <f>J10*L10</f>
@@ -5302,12 +6312,12 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Prateleira sobre a mesa</t>
+          <t>Nichos iluminados 3× (cabeceira)</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>Prateleira lâmina natural 170×25 c/ LED embutido, h = 1,95 m</t>
+          <t>Lâmina natural freijó, fundo preto, LED embutido</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -5322,7 +6332,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>170 × 25 × 3</t>
+          <t>3 × (24 × 26 × 16)</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
@@ -5345,11 +6355,11 @@
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>vb</t>
         </is>
       </c>
       <c r="L11" s="15" t="n">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="M11" s="16">
         <f>J11*L11</f>
@@ -6479,27 +7489,27 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Mão de obra de pintura</t>
+          <t>Luminária de mesa articulada</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Pintor c/ preparo completo (paredes + teto)</t>
+          <t>Luminária articulada preta, E27, lâmpada 2700 K</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Profissional local</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>Faixa R$ 15–35/m² simples; R$ 35–60/m² com preparo (Lar Pontual) — https://larpontual.com.br/portal/preco-de-pintor-por-m2</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
@@ -6522,17 +7532,16 @@
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="J30" s="14">
-        <f>area_pintura_total</f>
-        <v/>
+      <c r="J30" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L30" s="15" t="n">
-        <v>55</v>
+        <v>192</v>
       </c>
       <c r="M30" s="16">
         <f>J30*L30</f>
@@ -6542,27 +7551,27 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Instalação da iluminação</t>
+          <t>Suporte de headphone</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Montagem das fitas/perfis/fontes (marceneiro ou eletricista)</t>
+          <t>Suporte de mesa em metal preto</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Profissional local</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>Estimativa</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
@@ -6590,11 +7599,11 @@
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L31" s="15" t="n">
-        <v>400</v>
+        <v>96</v>
       </c>
       <c r="M31" s="16">
         <f>J31*L31</f>
@@ -6604,27 +7613,27 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Serviços</t>
+          <t>Decoração (opcional)</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Frete e taxas de importação</t>
+          <t>Quadros P&amp;B (3 na parede + 2 na prateleira)</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Reserva (Amazon Global pode ter impostos)</t>
+          <t>Impressões P&amp;B 40×55, 2× 36×26, 20×25, 15×20 c/ moldura preta e passe-partout</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>A pesquisar</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>Estimativa</t>
+          <t>Estimativa (preço não pesquisado)</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
@@ -6652,75 +7661,571 @@
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
-          <t>vb</t>
+          <t>un</t>
         </is>
       </c>
       <c r="L32" s="15" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="M32" s="16">
         <f>J32*L32</f>
         <v/>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Planta pendente</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Vaso cerâmica preta Ø18 + suporte de corda + samambaia + gancho de teto</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L33" s="15" t="n">
+        <v>192</v>
+      </c>
+      <c r="M33" s="16">
+        <f>J33*L33</f>
+        <v/>
+      </c>
+    </row>
     <row r="34">
-      <c r="L34" s="4" t="inlineStr">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Objetos dos nichos</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Vaso cerâmica + elefante em madeira + escultura de baleia (~15 cm)</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J34" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>320</v>
+      </c>
+      <c r="M34" s="16">
+        <f>J34*L34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Plantas da prateleira</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Vaso médio c/ planta + suculenta</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L35" s="15" t="n">
+        <v>160</v>
+      </c>
+      <c r="M35" s="16">
+        <f>J35*L35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Relógio LED de prateleira</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Relógio digital LED 12 cm</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J36" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>112</v>
+      </c>
+      <c r="M36" s="16">
+        <f>J36*L36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Decoração (opcional)</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Caneca e acessórios de mesa</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Caneca de cerâmica + porta-lápis</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>A pesquisar</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa (preço não pesquisado)</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J37" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="L37" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="M37" s="16">
+        <f>J37*L37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Mão de obra de pintura</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Pintor c/ preparo completo (paredes + teto)</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Profissional local</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Faixa R$ 15–35/m² simples; R$ 35–60/m² com preparo (Lar Pontual) — https://larpontual.com.br/portal/preco-de-pintor-por-m2</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J38" s="14">
+        <f>area_pintura_total</f>
+        <v/>
+      </c>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="M38" s="16">
+        <f>J38*L38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Instalação da iluminação</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Montagem das fitas/perfis/fontes (marceneiro ou eletricista)</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Profissional local</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J39" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="L39" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="M39" s="16">
+        <f>J39*L39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Frete e taxas de importação</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Reserva (Amazon Global pode ter impostos)</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>vb</t>
+        </is>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>450</v>
+      </c>
+      <c r="M40" s="16">
+        <f>J40*L40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="L42" s="4" t="inlineStr">
         <is>
           <t>Subtotal itens</t>
         </is>
       </c>
-      <c r="M34" s="6">
-        <f>SUM(M4:M32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="L35" s="4" t="inlineStr">
+      <c r="M42" s="6">
+        <f>SUM(M4:M40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="L43" s="4" t="inlineStr">
         <is>
           <t>Reserva para imprevistos</t>
         </is>
       </c>
-      <c r="M35" s="6">
-        <f>M34*contingencia</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="L36" s="4" t="inlineStr">
+      <c r="M43" s="6">
+        <f>M42*contingencia</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="L44" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="M36" s="6">
-        <f>M34+M35</f>
+      <c r="M44" s="6">
+        <f>M42+M43</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M32"/>
+  <autoFilter ref="A3:M40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6732,7 +8237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7489,20 +8994,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>n_verticais</t>
+          <t>led_nichos</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nº de perfis verticais (Econômico/Equilibrado)</t>
+          <t>LED dos 3 nichos (3 × 0,24)</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>1</v>
+        <v>0.72</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7514,72 +9019,71 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>perda_led</t>
+          <t>n_verticais</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Sobra de corte da fita</t>
-        </is>
-      </c>
-      <c r="C33" s="19" t="n">
-        <v>0.1</v>
+          <t>Nº de perfis verticais (Econômico/Equilibrado)</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>1</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>un</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Premissa</t>
+          <t>Projeto</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>metros_led</t>
+          <t>perda_led</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Metros de fita LED</t>
-        </is>
-      </c>
-      <c r="C34" s="18">
-        <f>(led_prateleira+led_vertical*n_verticais)*(1+perda_led)</f>
-        <v/>
+          <t>Sobra de corte da fita</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>0.1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Calculada</t>
+          <t>Premissa</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>rolos_led</t>
+          <t>metros_led</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Rolos de 5 m</t>
+          <t>Metros de fita LED</t>
         </is>
       </c>
       <c r="C35" s="18">
-        <f>ROUNDUP(metros_led/5,0)</f>
+        <f>(led_prateleira+led_vertical*n_verticais+led_nichos)*(1+perda_led)</f>
         <v/>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7591,21 +9095,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>barras_perfil</t>
+          <t>rolos_led</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Barras de perfil de 2 m</t>
+          <t>Rolos de 5 m</t>
         </is>
       </c>
       <c r="C36" s="18">
-        <f>ROUNDUP(led_prateleira/2,0)+n_verticais*ROUNDUP(led_vertical/2,0)</f>
+        <f>ROUNDUP(metros_led/5,0)</f>
         <v/>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>barra</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7617,72 +9121,72 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>n_verticais_prem</t>
+          <t>barras_perfil</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Nº de perfis verticais — Premium</t>
-        </is>
-      </c>
-      <c r="C37" s="17" t="n">
-        <v>2</v>
+          <t>Barras de perfil de 2 m</t>
+        </is>
+      </c>
+      <c r="C37" s="18">
+        <f>ROUNDUP(led_prateleira/2,0)+n_verticais*ROUNDUP(led_vertical/2,0)</f>
+        <v/>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>barra</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Projeto</t>
+          <t>Calculada</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>metros_led_prem</t>
+          <t>n_verticais_prem</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Metros de fita LED — Premium</t>
-        </is>
-      </c>
-      <c r="C38" s="18">
-        <f>(led_prateleira+led_vertical*n_verticais_prem)*(1+perda_led)</f>
-        <v/>
+          <t>Nº de perfis verticais — Premium</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="n">
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>un</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Calculada</t>
+          <t>Projeto</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>rolos_led_prem</t>
+          <t>metros_led_prem</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Rolos de 5 m — Premium</t>
+          <t>Metros de fita LED — Premium</t>
         </is>
       </c>
       <c r="C39" s="18">
-        <f>ROUNDUP(metros_led_prem/5,0)</f>
+        <f>(led_prateleira+led_vertical*n_verticais_prem+led_nichos)*(1+perda_led)</f>
         <v/>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7694,21 +9198,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>barras_perfil_prem</t>
+          <t>rolos_led_prem</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Barras de perfil de 2 m — Premium</t>
+          <t>Rolos de 5 m — Premium</t>
         </is>
       </c>
       <c r="C40" s="18">
-        <f>ROUNDUP(led_prateleira/2,0)+n_verticais_prem*ROUNDUP(led_vertical/2,0)</f>
+        <f>ROUNDUP(metros_led_prem/5,0)</f>
         <v/>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>barra</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -7720,23 +9224,49 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>barras_perfil_prem</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Barras de perfil de 2 m — Premium</t>
+        </is>
+      </c>
+      <c r="C41" s="18">
+        <f>ROUNDUP(led_prateleira/2,0)+n_verticais_prem*ROUNDUP(led_vertical/2,0)</f>
+        <v/>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Calculada</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>contingencia</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Reserva para imprevistos</t>
         </is>
       </c>
-      <c r="C41" s="19" t="n">
+      <c r="C42" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Premissa</t>
         </is>

</xml_diff>

<commit_message>
Revisão: planta de iluminação com L5/L6, legenda dos gráficos, notas e pendências
- Planta de iluminação: LED dos nichos (L5), luminária de mesa (L6), L3 no eixo novo
  dos monitores e carga da fonte 24 V
- planta_mobiliada.png (cópia antiga com PC suspenso) atualizada
- Gráficos do orçamento: legenda em 2 linhas (cortava "Reserva 10%")
- Notas da planilha (nichos, decoração estimada, PC no tampo) e novas pendências

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M4fUn4zoGcBfLLrM7oKPYT
</commit_message>
<xml_diff>
--- a/PROJETO_QUARTO_ESCRITORIO/04_ORCAMENTO/orcamento_completo.xlsx
+++ b/PROJETO_QUARTO_ESCRITORIO/04_ORCAMENTO/orcamento_completo.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -832,12 +832,26 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>• Marcenaria (ripado, tampo, prateleira) e mão de obra = estimativas por faixa de mercado; pedir 3 orçamentos locais.</t>
+          <t>• Marcenaria (ripado, tampo, prateleira, nichos) e mão de obra = estimativas por faixa de mercado; pedir 3 orçamentos locais.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>• Decoração (opcional): preços estimados, não pesquisados (loja bloqueada na sessão de 31/10/2026). Pesquisar antes de comprar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>• PC: fica sobre o tampo (suporte de gabinete removido em 31/10/2026). Monitores, PC e notebook são do usuário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>• Premium: a estrutura Marsail é vendida pela Amazon Global (importação); prazo e impostos podem variar.</t>
         </is>

</xml_diff>